<commit_message>
Add training results logging and model output paths for XGBoost classification
</commit_message>
<xml_diff>
--- a/confusion_matrix.xlsx
+++ b/confusion_matrix.xlsx
@@ -460,25 +460,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
         <v>0</v>
       </c>
       <c r="G2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -488,25 +488,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
         <v>101</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -522,10 +522,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -534,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5">
@@ -544,10 +544,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
         <v>0</v>
@@ -556,13 +556,13 @@
         <v>110</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -581,16 +581,16 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="F6" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="G6" t="n">
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -600,22 +600,22 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -631,13 +631,13 @@
         <v>0</v>
       </c>
       <c r="C8" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F8" t="n">
         <v>4</v>

</xml_diff>

<commit_message>
Update XGBoost classification model outputs and training history files
</commit_message>
<xml_diff>
--- a/confusion_matrix.xlsx
+++ b/confusion_matrix.xlsx
@@ -460,25 +460,25 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
         <v>3</v>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-      <c r="E2" t="n">
-        <v>0</v>
-      </c>
-      <c r="F2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -488,25 +488,25 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
+        <v>5</v>
+      </c>
+      <c r="H3" t="n">
         <v>3</v>
-      </c>
-      <c r="H3" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="4">
@@ -522,10 +522,10 @@
         <v>0</v>
       </c>
       <c r="D4" t="n">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="E4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -534,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -544,25 +544,25 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F5" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" t="n">
+        <v>4</v>
+      </c>
+      <c r="H5" t="n">
         <v>1</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -581,16 +581,16 @@
         <v>0</v>
       </c>
       <c r="E6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>119</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
         <v>1</v>
-      </c>
-      <c r="F6" t="n">
-        <v>117</v>
-      </c>
-      <c r="G6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="7">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C7" t="n">
         <v>0</v>
@@ -609,13 +609,13 @@
         <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -634,19 +634,19 @@
         <v>6</v>
       </c>
       <c r="D8" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
       <c r="F8" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
   </sheetData>

</xml_diff>